<commit_message>
Finalize project for deployment
</commit_message>
<xml_diff>
--- a/templates/Agile_Template_Filled.xlsx
+++ b/templates/Agile_Template_Filled.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc20060aec94d36e/Desktop/Multi-AI-Agent-Coding-Assistant - Copy(freebuff)/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bc20060aec94d36e/Desktop/Multi-AI-Agent-Coding-Assistant/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="11_35405060270B16A5D1AF267B1094433D5596BCCE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE2049BD-3765-44CE-9476-DC0B048E95FC}"/>
+  <xr:revisionPtr revIDLastSave="194" documentId="11_754690141E3C98E11DCBAA6B96695E6566B1059D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0DB483C-9A97-49DF-AE99-CF536F9C0842}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="775" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="775" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product Backlog" sheetId="1" r:id="rId1"/>
@@ -286,7 +286,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="607" uniqueCount="283">
   <si>
     <t>NOTES:  Task sizing should be between 0.5 to 12 hours</t>
   </si>
@@ -498,63 +498,63 @@
     <t>Redesign UI - theme.py design system, login screen, sidebar</t>
   </si>
   <si>
+    <t>US-012</t>
+  </si>
+  <si>
+    <t>T-022</t>
+  </si>
+  <si>
+    <t>Workspace quick actions (ask-first) + drag-and-drop upload zone</t>
+  </si>
+  <si>
+    <t>02-Aug-2026</t>
+  </si>
+  <si>
+    <t>US-013</t>
+  </si>
+  <si>
+    <t>T-023</t>
+  </si>
+  <si>
+    <t>Private My Files library - CRUD, preview, search, filter</t>
+  </si>
+  <si>
+    <t>04-Aug-2026</t>
+  </si>
+  <si>
+    <t>US-014</t>
+  </si>
+  <si>
+    <t>T-024</t>
+  </si>
+  <si>
+    <t>Analytics dashboard - exact KPI cards + daily usage charts</t>
+  </si>
+  <si>
     <t>03-Aug-2026</t>
   </si>
   <si>
-    <t>US-012</t>
-  </si>
-  <si>
-    <t>T-022</t>
-  </si>
-  <si>
-    <t>Workspace quick actions (ask-first) + drag-and-drop upload zone</t>
-  </si>
-  <si>
-    <t>02-Aug-2026</t>
-  </si>
-  <si>
-    <t>04-Aug-2026</t>
-  </si>
-  <si>
-    <t>US-013</t>
-  </si>
-  <si>
-    <t>T-023</t>
-  </si>
-  <si>
-    <t>Private My Files library - CRUD, preview, search, filter</t>
-  </si>
-  <si>
-    <t>US-014</t>
-  </si>
-  <si>
-    <t>T-024</t>
-  </si>
-  <si>
-    <t>Analytics dashboard - exact KPI cards + daily usage charts</t>
+    <t>US-015</t>
+  </si>
+  <si>
+    <t>T-025</t>
+  </si>
+  <si>
+    <t>Chat History search/export + Settings + Profile + legal pages</t>
+  </si>
+  <si>
+    <t>US-016</t>
+  </si>
+  <si>
+    <t>T-026</t>
+  </si>
+  <si>
+    <t>Fix file uploader duplicate-save + upload dedupe</t>
   </si>
   <si>
     <t>05-Aug-2026</t>
   </si>
   <si>
-    <t>US-015</t>
-  </si>
-  <si>
-    <t>T-025</t>
-  </si>
-  <si>
-    <t>Chat History search/export + Settings + Profile + legal pages</t>
-  </si>
-  <si>
-    <t>US-016</t>
-  </si>
-  <si>
-    <t>T-026</t>
-  </si>
-  <si>
-    <t>Fix file uploader duplicate-save + upload dedupe</t>
-  </si>
-  <si>
     <t>T-027</t>
   </si>
   <si>
@@ -567,6 +567,114 @@
     <t>Exact analytics KPIs - success rate + conversation counts</t>
   </si>
   <si>
+    <t>SPRINT  4  BACKLOG</t>
+  </si>
+  <si>
+    <t>US-017</t>
+  </si>
+  <si>
+    <t>T-029</t>
+  </si>
+  <si>
+    <t>Google OAuth - login page button, callback, session restore</t>
+  </si>
+  <si>
+    <t>US-023</t>
+  </si>
+  <si>
+    <t>T-030</t>
+  </si>
+  <si>
+    <t>REST API server (api/server.py) + monitoring metrics + deployment configs</t>
+  </si>
+  <si>
+    <t>US-018</t>
+  </si>
+  <si>
+    <t>T-031</t>
+  </si>
+  <si>
+    <t>Intent-based routing cleanup - project vs code analysis, error-handling follow-ups, planner pinning</t>
+  </si>
+  <si>
+    <t>US-019</t>
+  </si>
+  <si>
+    <t>T-032</t>
+  </si>
+  <si>
+    <t>Project ZIP: extract, attach, Project Analyzer reads the actual files (first turn)</t>
+  </si>
+  <si>
+    <t>T-033</t>
+  </si>
+  <si>
+    <t>No-ZIP safety guard - never scan the assistant workspace, ask for the project</t>
+  </si>
+  <si>
+    <t>US-020</t>
+  </si>
+  <si>
+    <t>T-034</t>
+  </si>
+  <si>
+    <t>Agent output cleanup - strip &lt;think&gt; blocks, concise reviewer/docs/coding prompts</t>
+  </si>
+  <si>
+    <t>T-035</t>
+  </si>
+  <si>
+    <t>Static metrics hidden unless explicitly requested</t>
+  </si>
+  <si>
+    <t>US-021</t>
+  </si>
+  <si>
+    <t>T-036</t>
+  </si>
+  <si>
+    <t>UI polish - table/code overflow CSS, model selector internal, no internal metadata</t>
+  </si>
+  <si>
+    <t>US-024</t>
+  </si>
+  <si>
+    <t>T-037</t>
+  </si>
+  <si>
+    <t>Graceful error handling for provider rate limits and tool failures</t>
+  </si>
+  <si>
+    <t>US-022</t>
+  </si>
+  <si>
+    <t>T-038</t>
+  </si>
+  <si>
+    <t>Experimental media/vision support evaluated and removed entirely (menu, model, tests)</t>
+  </si>
+  <si>
+    <t>T-039</t>
+  </si>
+  <si>
+    <t>Simplify the + menu to a single Upload File action; ZIP archives are still extracted and analyzed as projects</t>
+  </si>
+  <si>
+    <t>T-040</t>
+  </si>
+  <si>
+    <t>Follow-up routing fixes - error-handling verbs, planner expansion, improvement questions</t>
+  </si>
+  <si>
+    <t>US-025</t>
+  </si>
+  <si>
+    <t>T-041</t>
+  </si>
+  <si>
+    <t>Regression tests for routing, context, file/project upload, UI (276 passing)</t>
+  </si>
+  <si>
     <t>Planned Sprint</t>
   </si>
   <si>
@@ -657,6 +765,36 @@
     <t>As a user, I want reliable file handling - no duplicate uploads, correct routing of 'analyse it'/ 'review it' / 'generate documentation' with attached files, and accurate KPIs - so that the product behaves consistently.</t>
   </si>
   <si>
+    <t>Sprint 4</t>
+  </si>
+  <si>
+    <t>As a user, I want to sign in with my Google account so that I can use the application without creating a separate account.</t>
+  </si>
+  <si>
+    <t>As a user, I want requests routed by my actual intent (coding, debugging, documentation, planning, analysis) and follow-up questions to keep the same conversation and file/project context.</t>
+  </si>
+  <si>
+    <t>As a user, I want a project ZIP analyzed, reviewed, planned and documented from its ACTUAL extracted files, with a friendly upload prompt when no project is available.</t>
+  </si>
+  <si>
+    <t>As a user, I want simple, readable agent output - concise reviews, clean documentation, no static metrics or AI filler, and no internal reasoning blocks.</t>
+  </si>
+  <si>
+    <t>As a user, I want a clean GPT-like UI where markdown tables and code stay inside the chat bubble, internal model/token details stay hidden, and the + menu only shows useful actions.</t>
+  </si>
+  <si>
+    <t>As a product decision, remove experimental media/vision support so the app stays focused on code, files and projects.</t>
+  </si>
+  <si>
+    <t>As an operator, I want a standalone REST API with monitoring metrics and deployment configuration (Docker, Render, Railway) so the assistant can be deployed.</t>
+  </si>
+  <si>
+    <t>As a user, I want friendly error messages when an LLM call, tool or file fails - never a raw traceback - with the real error logged for debugging.</t>
+  </si>
+  <si>
+    <t>As a stakeholder, I want a comprehensive regression suite (276 tests) covering routing, follow-up context, file/project upload and the UI.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sprint </t>
   </si>
   <si>
@@ -756,6 +894,48 @@
     <t>Made all dashboard numbers derive from real records.</t>
   </si>
   <si>
+    <t>A request with attached content was routed by a keyword ('analyze') instead of the actual subject, so the attachment was ignored.</t>
+  </si>
+  <si>
+    <t>Added subject-aware routing guards; the experimental media feature was later removed per product decision.</t>
+  </si>
+  <si>
+    <t>"Analyze this project" with an uploaded ZIP reached the Code Analysis Agent instead of Project Analyzer.</t>
+  </si>
+  <si>
+    <t>Added a project-subject guard so project requests reach the Project Analyzer.</t>
+  </si>
+  <si>
+    <t>"Analyze this Python code" with a pasted snippet and attached project was misrouted to Documentation.</t>
+  </si>
+  <si>
+    <t>Deterministic analyze-to-code-analysis pin before the LLM; matching uses only the user's own words.</t>
+  </si>
+  <si>
+    <t>Groq vision output showed raw &lt;think&gt; reasoning and truncated answers.</t>
+  </si>
+  <si>
+    <t>Stripped think blocks before display and before the empty check; raised the vision token budget.</t>
+  </si>
+  <si>
+    <t>"Also handle invalid non-numeric input" follow-up went to the Patch Tool with a hallucinated file.</t>
+  </si>
+  <si>
+    <t>Added error-handling follow-up verbs so it stays in the debugging conversation.</t>
+  </si>
+  <si>
+    <t>Markdown tables and long code extended outside the chat bubble.</t>
+  </si>
+  <si>
+    <t>Targeted CSS keeps tables wrapping and code scrolling inside the container.</t>
+  </si>
+  <si>
+    <t>Stale project report text leaked into new requests.</t>
+  </si>
+  <si>
+    <t>New topics strip previous-turn blocks; new attachments replace old context.</t>
+  </si>
+  <si>
     <t>SL #</t>
   </si>
   <si>
@@ -901,6 +1081,60 @@
   </si>
   <si>
     <t>Added routing fixes for attached-file analysis.</t>
+  </si>
+  <si>
+    <t>Keep deterministic routing pins for key intent verbs before trusting the LLM.</t>
+  </si>
+  <si>
+    <t>Routing on prompt wording alone without attachment/project context.</t>
+  </si>
+  <si>
+    <t>Verifying every workflow live in the UI before reporting it fixed.</t>
+  </si>
+  <si>
+    <t>Added deterministic overrides plus a 276-test regression suite.</t>
+  </si>
+  <si>
+    <t>Remove experimental features that add risk without user value.</t>
+  </si>
+  <si>
+    <t>Keeping two overlapping upload paths for the same project archive.</t>
+  </si>
+  <si>
+    <t>Keeping the + menu minimal - Upload File plus actions only.</t>
+  </si>
+  <si>
+    <t>Consolidated uploads into a single Upload File action; ZIP archives keep the project workflow.</t>
+  </si>
+  <si>
+    <t>Hide internal reasoning, metrics and model details from user output.</t>
+  </si>
+  <si>
+    <t>Letting the LLM classify without deterministic guards on follow-up context.</t>
+  </si>
+  <si>
+    <t>Keeping agent output simple, concise and proportional to the request.</t>
+  </si>
+  <si>
+    <t>Stripped think blocks, hid static metrics, cleaned reviewer/docs/coding prompts.</t>
+  </si>
+  <si>
+    <t>Day 42</t>
+  </si>
+  <si>
+    <t>Day 43</t>
+  </si>
+  <si>
+    <t>Day 44</t>
+  </si>
+  <si>
+    <t>Day 45</t>
+  </si>
+  <si>
+    <t>Day 46</t>
+  </si>
+  <si>
+    <t>Day 47</t>
   </si>
 </sst>
 </file>
@@ -1421,14 +1655,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="9" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1748,7 +1982,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.44140625" customWidth="1"/>
@@ -1761,25 +1995,25 @@
   <sheetData>
     <row r="1" spans="1:8" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
-        <v>93</v>
+        <v>129</v>
       </c>
       <c r="B1" s="18" t="s">
-        <v>94</v>
+        <v>130</v>
       </c>
       <c r="C1" s="19" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="19" t="s">
-        <v>95</v>
+        <v>131</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>96</v>
+        <v>132</v>
       </c>
       <c r="F1" s="19" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="G1" s="19" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
       <c r="H1" s="19" t="s">
         <v>8</v>
@@ -1787,45 +2021,45 @@
     </row>
     <row r="2" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C2" s="51" t="s">
         <v>25</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="E2" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>102</v>
+        <v>138</v>
       </c>
       <c r="G2" s="26" t="s">
         <v>28</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C3" s="27" t="s">
         <v>33</v>
       </c>
       <c r="D3" s="29" t="s">
-        <v>104</v>
+        <v>140</v>
       </c>
       <c r="E3" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F3" s="26" t="s">
         <v>25</v>
@@ -1834,24 +2068,24 @@
         <v>28</v>
       </c>
       <c r="H3" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C4" s="27" t="s">
         <v>37</v>
       </c>
       <c r="D4" s="29" t="s">
-        <v>105</v>
+        <v>141</v>
       </c>
       <c r="E4" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F4" s="26" t="s">
         <v>33</v>
@@ -1860,24 +2094,24 @@
         <v>28</v>
       </c>
       <c r="H4" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C5" s="27" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="29" t="s">
-        <v>106</v>
+        <v>142</v>
       </c>
       <c r="E5" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F5" s="26" t="s">
         <v>37</v>
@@ -1886,24 +2120,24 @@
         <v>28</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="25.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C6" s="27" t="s">
         <v>44</v>
       </c>
       <c r="D6" s="29" t="s">
-        <v>107</v>
+        <v>143</v>
       </c>
       <c r="E6" s="26" t="s">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="F6" s="26" t="s">
         <v>41</v>
@@ -1912,24 +2146,24 @@
         <v>28</v>
       </c>
       <c r="H6" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C7" s="27" t="s">
         <v>48</v>
       </c>
       <c r="D7" s="29" t="s">
-        <v>110</v>
+        <v>146</v>
       </c>
       <c r="E7" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F7" s="26" t="s">
         <v>41</v>
@@ -1938,24 +2172,24 @@
         <v>28</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C8" s="27" t="s">
         <v>51</v>
       </c>
       <c r="D8" s="29" t="s">
-        <v>111</v>
+        <v>147</v>
       </c>
       <c r="E8" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F8" s="26" t="s">
         <v>48</v>
@@ -1964,24 +2198,24 @@
         <v>28</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C9" s="27" t="s">
         <v>56</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>112</v>
+        <v>148</v>
       </c>
       <c r="E9" s="26" t="s">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="F9" s="26" t="s">
         <v>51</v>
@@ -1990,24 +2224,24 @@
         <v>28</v>
       </c>
       <c r="H9" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C10" s="27" t="s">
         <v>59</v>
       </c>
       <c r="D10" s="29" t="s">
-        <v>113</v>
+        <v>149</v>
       </c>
       <c r="E10" s="26" t="s">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="F10" s="26" t="s">
         <v>51</v>
@@ -2016,24 +2250,24 @@
         <v>28</v>
       </c>
       <c r="H10" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="25.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C11" s="27" t="s">
         <v>62</v>
       </c>
       <c r="D11" s="29" t="s">
-        <v>114</v>
+        <v>150</v>
       </c>
       <c r="E11" s="26" t="s">
-        <v>115</v>
+        <v>151</v>
       </c>
       <c r="F11" s="26" t="s">
         <v>59</v>
@@ -2042,24 +2276,24 @@
         <v>28</v>
       </c>
       <c r="H11" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C12" s="29" t="s">
         <v>67</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>117</v>
+        <v>153</v>
       </c>
       <c r="E12" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F12" s="26" t="s">
         <v>62</v>
@@ -2068,24 +2302,24 @@
         <v>28</v>
       </c>
       <c r="H12" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C13" s="50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D13" s="29" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="E13" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F13" s="26" t="s">
         <v>67</v>
@@ -2094,111 +2328,345 @@
         <v>28</v>
       </c>
       <c r="H13" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C14" s="27" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>119</v>
+        <v>155</v>
       </c>
       <c r="E14" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F14" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G14" s="26" t="s">
         <v>28</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D15" s="29" t="s">
-        <v>120</v>
+        <v>156</v>
       </c>
       <c r="E15" s="26" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
       <c r="F15" s="26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G15" s="26" t="s">
         <v>28</v>
       </c>
       <c r="H15" s="26" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="22.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C16" s="27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>121</v>
+        <v>157</v>
       </c>
       <c r="E16" s="26" t="s">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="F16" s="26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G16" s="26" t="s">
         <v>28</v>
       </c>
       <c r="H16" s="26" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" s="26" t="s">
+        <v>152</v>
+      </c>
+      <c r="C17" s="50" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F17" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C18" s="50" t="s">
+        <v>94</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>160</v>
+      </c>
+      <c r="E18" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F18" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="G18" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C19" s="50" t="s">
+        <v>100</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>161</v>
+      </c>
+      <c r="E19" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F19" s="26" t="s">
+        <v>94</v>
+      </c>
+      <c r="G19" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C20" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="E20" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F20" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="G20" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H20" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C21" s="50" t="s">
+        <v>108</v>
+      </c>
+      <c r="D21" s="29" t="s">
+        <v>163</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="F21" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="G21" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H21" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C22" s="50" t="s">
+        <v>113</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>164</v>
+      </c>
+      <c r="E22" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="F22" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="G22" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B23" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C23" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>165</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>151</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>108</v>
+      </c>
+      <c r="G23" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H23" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B24" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="50" t="s">
+        <v>97</v>
+      </c>
+      <c r="D24" s="29" t="s">
+        <v>166</v>
+      </c>
+      <c r="E24" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F24" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="G24" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H24" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="D25" s="29" t="s">
+        <v>167</v>
+      </c>
+      <c r="E25" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="F25" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="G25" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H25" s="26" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="B26" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="C26" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="E26" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="F26" s="26" t="s">
         <v>116</v>
       </c>
-      <c r="C17" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="D17" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="E17" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="F17" s="26" t="s">
-        <v>76</v>
-      </c>
-      <c r="G17" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="26" t="s">
-        <v>103</v>
+      <c r="G26" s="26" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="26" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2234,8 +2702,8 @@
     <col min="10" max="10" width="10.88671875" style="11" customWidth="1"/>
     <col min="11" max="11" width="10.33203125" style="11" customWidth="1"/>
     <col min="12" max="12" width="10.109375" style="11" customWidth="1"/>
-    <col min="13" max="20" width="9.109375" style="11" customWidth="1"/>
-    <col min="21" max="16384" width="9.109375" style="11"/>
+    <col min="13" max="22" width="9.109375" style="11" customWidth="1"/>
+    <col min="23" max="16384" width="9.109375" style="11"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -2266,10 +2734,10 @@
       <c r="W1" s="24"/>
     </row>
     <row r="2" spans="1:23" s="12" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="61" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="63" t="s">
+      <c r="A2" s="63" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="61" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="65" t="s">
@@ -2337,8 +2805,8 @@
       </c>
     </row>
     <row r="3" spans="1:23" s="12" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="62"/>
-      <c r="B3" s="64"/>
+      <c r="A3" s="64"/>
+      <c r="B3" s="62"/>
       <c r="C3" s="60"/>
       <c r="D3" s="60"/>
       <c r="E3" s="60"/>
@@ -2347,55 +2815,55 @@
       <c r="H3" s="60"/>
       <c r="I3" s="25">
         <f t="shared" ref="I3:W3" si="0">SUM(I5:I802)</f>
-        <v>114</v>
+        <v>199</v>
       </c>
       <c r="J3" s="25">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="K3" s="25">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="L3" s="25">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="M3" s="25">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="N3" s="25">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="O3" s="25">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="P3" s="25">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="Q3" s="25">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="R3" s="25">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="S3" s="25">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T3" s="25">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U3" s="25">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V3" s="25">
         <f t="shared" si="0"/>
@@ -3412,16 +3880,16 @@
     </row>
     <row r="20" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="34" t="s">
+      <c r="C20" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="34" t="s">
+      <c r="D20" s="14" t="s">
         <v>73</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>74</v>
       </c>
       <c r="E20" s="13">
         <v>46237</v>
@@ -3483,19 +3951,19 @@
     </row>
     <row r="21" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="B21" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="C21" s="34" t="s">
         <v>76</v>
-      </c>
-      <c r="B21" s="34" t="s">
-        <v>77</v>
-      </c>
-      <c r="C21" s="34" t="s">
-        <v>78</v>
       </c>
       <c r="D21" s="49">
         <v>46237</v>
       </c>
       <c r="E21" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F21" s="44" t="s">
         <v>28</v>
@@ -3554,16 +4022,16 @@
     </row>
     <row r="22" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B22" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="B22" s="34" t="s">
+      <c r="C22" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="D22" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="D22" s="14" t="s">
-        <v>70</v>
       </c>
       <c r="E22" s="13">
         <v>46238</v>
@@ -3625,16 +4093,16 @@
     </row>
     <row r="23" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B23" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="B23" s="34" t="s">
+      <c r="C23" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="C23" s="34" t="s">
-        <v>85</v>
-      </c>
       <c r="D23" s="14" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E23" s="13">
         <v>46239</v>
@@ -3696,19 +4164,19 @@
     </row>
     <row r="24" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="34" t="s">
         <v>86</v>
       </c>
-      <c r="B24" s="34" t="s">
+      <c r="C24" s="34" t="s">
         <v>87</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="D24" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" s="13" t="s">
         <v>88</v>
-      </c>
-      <c r="D24" s="14" t="s">
-        <v>75</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>82</v>
       </c>
       <c r="F24" s="44" t="s">
         <v>28</v>
@@ -3767,7 +4235,7 @@
     </row>
     <row r="25" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B25" s="34" t="s">
         <v>89</v>
@@ -3776,10 +4244,10 @@
         <v>90</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E25" s="13" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F25" s="44" t="s">
         <v>28</v>
@@ -3838,7 +4306,7 @@
     </row>
     <row r="26" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B26" s="34" t="s">
         <v>91</v>
@@ -3847,10 +4315,10 @@
         <v>92</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F26" s="44" t="s">
         <v>28</v>
@@ -3907,28 +4375,964 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:23" ht="29.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:23" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:23" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:23" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:23" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="20.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:23" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="56" t="s">
+        <v>93</v>
+      </c>
+      <c r="B27" s="57"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="57"/>
+      <c r="E27" s="57"/>
+      <c r="F27" s="57"/>
+      <c r="G27" s="57"/>
+      <c r="H27" s="57"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="57"/>
+      <c r="K27" s="57"/>
+      <c r="L27" s="57"/>
+      <c r="M27" s="57"/>
+      <c r="N27" s="57"/>
+      <c r="O27" s="57"/>
+      <c r="P27" s="57"/>
+      <c r="Q27" s="57"/>
+      <c r="R27" s="57"/>
+      <c r="S27" s="57"/>
+      <c r="T27" s="57"/>
+      <c r="U27" s="57"/>
+      <c r="V27" s="57"/>
+      <c r="W27" s="58"/>
+    </row>
+    <row r="28" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="B28" s="34" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="D28" s="49">
+        <v>46240</v>
+      </c>
+      <c r="E28" s="13">
+        <v>46241</v>
+      </c>
+      <c r="F28" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H28" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I28" s="15">
+        <v>8</v>
+      </c>
+      <c r="J28" s="15">
+        <v>1</v>
+      </c>
+      <c r="K28" s="15">
+        <v>1</v>
+      </c>
+      <c r="L28" s="15">
+        <v>1</v>
+      </c>
+      <c r="M28" s="16">
+        <v>1</v>
+      </c>
+      <c r="N28" s="16">
+        <v>1</v>
+      </c>
+      <c r="O28" s="16">
+        <v>1</v>
+      </c>
+      <c r="P28" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q28" s="16">
+        <v>1</v>
+      </c>
+      <c r="R28" s="16">
+        <v>0</v>
+      </c>
+      <c r="S28" s="16">
+        <v>0</v>
+      </c>
+      <c r="T28" s="16">
+        <v>0</v>
+      </c>
+      <c r="U28" s="16">
+        <v>0</v>
+      </c>
+      <c r="V28" s="16">
+        <v>0</v>
+      </c>
+      <c r="W28" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" ht="38.4" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C29" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="D29" s="49">
+        <v>46240</v>
+      </c>
+      <c r="E29" s="13">
+        <v>46243</v>
+      </c>
+      <c r="F29" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G29" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H29" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I29" s="15">
+        <v>12</v>
+      </c>
+      <c r="J29" s="15">
+        <v>1</v>
+      </c>
+      <c r="K29" s="15">
+        <v>1</v>
+      </c>
+      <c r="L29" s="15">
+        <v>1</v>
+      </c>
+      <c r="M29" s="16">
+        <v>1</v>
+      </c>
+      <c r="N29" s="16">
+        <v>1</v>
+      </c>
+      <c r="O29" s="16">
+        <v>1</v>
+      </c>
+      <c r="P29" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q29" s="16">
+        <v>1</v>
+      </c>
+      <c r="R29" s="16">
+        <v>1</v>
+      </c>
+      <c r="S29" s="16">
+        <v>1</v>
+      </c>
+      <c r="T29" s="16">
+        <v>1</v>
+      </c>
+      <c r="U29" s="16">
+        <v>1</v>
+      </c>
+      <c r="V29" s="16">
+        <v>0</v>
+      </c>
+      <c r="W29" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" ht="58.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B30" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="C30" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="D30" s="49">
+        <v>46242</v>
+      </c>
+      <c r="E30" s="13">
+        <v>46244</v>
+      </c>
+      <c r="F30" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G30" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H30" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I30" s="15">
+        <v>10</v>
+      </c>
+      <c r="J30" s="15">
+        <v>1</v>
+      </c>
+      <c r="K30" s="15">
+        <v>1</v>
+      </c>
+      <c r="L30" s="15">
+        <v>1</v>
+      </c>
+      <c r="M30" s="16">
+        <v>1</v>
+      </c>
+      <c r="N30" s="16">
+        <v>1</v>
+      </c>
+      <c r="O30" s="16">
+        <v>1</v>
+      </c>
+      <c r="P30" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="16">
+        <v>1</v>
+      </c>
+      <c r="R30" s="16">
+        <v>1</v>
+      </c>
+      <c r="S30" s="16">
+        <v>1</v>
+      </c>
+      <c r="T30" s="16">
+        <v>0</v>
+      </c>
+      <c r="U30" s="16">
+        <v>0</v>
+      </c>
+      <c r="V30" s="16">
+        <v>0</v>
+      </c>
+      <c r="W30" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" ht="36.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="B31" s="34" t="s">
+        <v>104</v>
+      </c>
+      <c r="C31" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="D31" s="49">
+        <v>46244</v>
+      </c>
+      <c r="E31" s="13">
+        <v>46245</v>
+      </c>
+      <c r="F31" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G31" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H31" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I31" s="15">
+        <v>9</v>
+      </c>
+      <c r="J31" s="15">
+        <v>1</v>
+      </c>
+      <c r="K31" s="15">
+        <v>1</v>
+      </c>
+      <c r="L31" s="15">
+        <v>1</v>
+      </c>
+      <c r="M31" s="16">
+        <v>1</v>
+      </c>
+      <c r="N31" s="16">
+        <v>1</v>
+      </c>
+      <c r="O31" s="16">
+        <v>1</v>
+      </c>
+      <c r="P31" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q31" s="16">
+        <v>1</v>
+      </c>
+      <c r="R31" s="16">
+        <v>1</v>
+      </c>
+      <c r="S31" s="16">
+        <v>0</v>
+      </c>
+      <c r="T31" s="16">
+        <v>0</v>
+      </c>
+      <c r="U31" s="16">
+        <v>0</v>
+      </c>
+      <c r="V31" s="16">
+        <v>0</v>
+      </c>
+      <c r="W31" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="32" t="s">
+        <v>103</v>
+      </c>
+      <c r="B32" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="49">
+        <v>46245</v>
+      </c>
+      <c r="E32" s="13">
+        <v>46245</v>
+      </c>
+      <c r="F32" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G32" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H32" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I32" s="15">
+        <v>3</v>
+      </c>
+      <c r="J32" s="15">
+        <v>1</v>
+      </c>
+      <c r="K32" s="15">
+        <v>1</v>
+      </c>
+      <c r="L32" s="15">
+        <v>1</v>
+      </c>
+      <c r="M32" s="16">
+        <v>0</v>
+      </c>
+      <c r="N32" s="16">
+        <v>0</v>
+      </c>
+      <c r="O32" s="16">
+        <v>0</v>
+      </c>
+      <c r="P32" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="16">
+        <v>0</v>
+      </c>
+      <c r="R32" s="16">
+        <v>0</v>
+      </c>
+      <c r="S32" s="16">
+        <v>0</v>
+      </c>
+      <c r="T32" s="16">
+        <v>0</v>
+      </c>
+      <c r="U32" s="16">
+        <v>0</v>
+      </c>
+      <c r="V32" s="16">
+        <v>0</v>
+      </c>
+      <c r="W32" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" ht="46.8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>110</v>
+      </c>
+      <c r="D33" s="49">
+        <v>46245</v>
+      </c>
+      <c r="E33" s="13">
+        <v>46247</v>
+      </c>
+      <c r="F33" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G33" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H33" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I33" s="15">
+        <v>8</v>
+      </c>
+      <c r="J33" s="15">
+        <v>1</v>
+      </c>
+      <c r="K33" s="15">
+        <v>1</v>
+      </c>
+      <c r="L33" s="15">
+        <v>1</v>
+      </c>
+      <c r="M33" s="16">
+        <v>1</v>
+      </c>
+      <c r="N33" s="16">
+        <v>1</v>
+      </c>
+      <c r="O33" s="16">
+        <v>1</v>
+      </c>
+      <c r="P33" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="16">
+        <v>1</v>
+      </c>
+      <c r="R33" s="16">
+        <v>0</v>
+      </c>
+      <c r="S33" s="16">
+        <v>0</v>
+      </c>
+      <c r="T33" s="16">
+        <v>0</v>
+      </c>
+      <c r="U33" s="16">
+        <v>0</v>
+      </c>
+      <c r="V33" s="16">
+        <v>0</v>
+      </c>
+      <c r="W33" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" ht="33.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B34" s="34" t="s">
+        <v>111</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>112</v>
+      </c>
+      <c r="D34" s="49">
+        <v>46247</v>
+      </c>
+      <c r="E34" s="13">
+        <v>46247</v>
+      </c>
+      <c r="F34" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H34" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I34" s="15">
+        <v>3</v>
+      </c>
+      <c r="J34" s="15">
+        <v>1</v>
+      </c>
+      <c r="K34" s="15">
+        <v>1</v>
+      </c>
+      <c r="L34" s="15">
+        <v>1</v>
+      </c>
+      <c r="M34" s="16">
+        <v>0</v>
+      </c>
+      <c r="N34" s="16">
+        <v>0</v>
+      </c>
+      <c r="O34" s="16">
+        <v>0</v>
+      </c>
+      <c r="P34" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="16">
+        <v>0</v>
+      </c>
+      <c r="R34" s="16">
+        <v>0</v>
+      </c>
+      <c r="S34" s="16">
+        <v>0</v>
+      </c>
+      <c r="T34" s="16">
+        <v>0</v>
+      </c>
+      <c r="U34" s="16">
+        <v>0</v>
+      </c>
+      <c r="V34" s="16">
+        <v>0</v>
+      </c>
+      <c r="W34" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" ht="44.4" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="C35" s="34" t="s">
+        <v>115</v>
+      </c>
+      <c r="D35" s="49">
+        <v>46247</v>
+      </c>
+      <c r="E35" s="13">
+        <v>46248</v>
+      </c>
+      <c r="F35" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G35" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H35" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I35" s="15">
+        <v>6</v>
+      </c>
+      <c r="J35" s="15">
+        <v>1</v>
+      </c>
+      <c r="K35" s="15">
+        <v>1</v>
+      </c>
+      <c r="L35" s="15">
+        <v>1</v>
+      </c>
+      <c r="M35" s="16">
+        <v>1</v>
+      </c>
+      <c r="N35" s="16">
+        <v>1</v>
+      </c>
+      <c r="O35" s="16">
+        <v>1</v>
+      </c>
+      <c r="P35" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="16">
+        <v>0</v>
+      </c>
+      <c r="R35" s="16">
+        <v>0</v>
+      </c>
+      <c r="S35" s="16">
+        <v>0</v>
+      </c>
+      <c r="T35" s="16">
+        <v>0</v>
+      </c>
+      <c r="U35" s="16">
+        <v>0</v>
+      </c>
+      <c r="V35" s="16">
+        <v>0</v>
+      </c>
+      <c r="W35" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" ht="35.4" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="32" t="s">
+        <v>116</v>
+      </c>
+      <c r="B36" s="34" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="34" t="s">
+        <v>118</v>
+      </c>
+      <c r="D36" s="49">
+        <v>46248</v>
+      </c>
+      <c r="E36" s="13">
+        <v>46248</v>
+      </c>
+      <c r="F36" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G36" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H36" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I36" s="15">
+        <v>3</v>
+      </c>
+      <c r="J36" s="15">
+        <v>1</v>
+      </c>
+      <c r="K36" s="15">
+        <v>1</v>
+      </c>
+      <c r="L36" s="15">
+        <v>1</v>
+      </c>
+      <c r="M36" s="16">
+        <v>0</v>
+      </c>
+      <c r="N36" s="16">
+        <v>0</v>
+      </c>
+      <c r="O36" s="16">
+        <v>0</v>
+      </c>
+      <c r="P36" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="16">
+        <v>0</v>
+      </c>
+      <c r="R36" s="16">
+        <v>0</v>
+      </c>
+      <c r="S36" s="16">
+        <v>0</v>
+      </c>
+      <c r="T36" s="16">
+        <v>0</v>
+      </c>
+      <c r="U36" s="16">
+        <v>0</v>
+      </c>
+      <c r="V36" s="16">
+        <v>0</v>
+      </c>
+      <c r="W36" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" ht="52.8" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="32" t="s">
+        <v>119</v>
+      </c>
+      <c r="B37" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="C37" s="34" t="s">
+        <v>121</v>
+      </c>
+      <c r="D37" s="49">
+        <v>46248</v>
+      </c>
+      <c r="E37" s="13">
+        <v>46249</v>
+      </c>
+      <c r="F37" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G37" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H37" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I37" s="15">
+        <v>8</v>
+      </c>
+      <c r="J37" s="15">
+        <v>1</v>
+      </c>
+      <c r="K37" s="15">
+        <v>1</v>
+      </c>
+      <c r="L37" s="15">
+        <v>1</v>
+      </c>
+      <c r="M37" s="16">
+        <v>1</v>
+      </c>
+      <c r="N37" s="16">
+        <v>1</v>
+      </c>
+      <c r="O37" s="16">
+        <v>1</v>
+      </c>
+      <c r="P37" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q37" s="16">
+        <v>1</v>
+      </c>
+      <c r="R37" s="16">
+        <v>0</v>
+      </c>
+      <c r="S37" s="16">
+        <v>0</v>
+      </c>
+      <c r="T37" s="16">
+        <v>0</v>
+      </c>
+      <c r="U37" s="16">
+        <v>0</v>
+      </c>
+      <c r="V37" s="16">
+        <v>0</v>
+      </c>
+      <c r="W37" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" ht="46.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="32" t="s">
+        <v>113</v>
+      </c>
+      <c r="B38" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="C38" s="34" t="s">
+        <v>123</v>
+      </c>
+      <c r="D38" s="49">
+        <v>46250</v>
+      </c>
+      <c r="E38" s="13">
+        <v>46250</v>
+      </c>
+      <c r="F38" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G38" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H38" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I38" s="15">
+        <v>2</v>
+      </c>
+      <c r="J38" s="15">
+        <v>1</v>
+      </c>
+      <c r="K38" s="15">
+        <v>1</v>
+      </c>
+      <c r="L38" s="15">
+        <v>0</v>
+      </c>
+      <c r="M38" s="16">
+        <v>0</v>
+      </c>
+      <c r="N38" s="16">
+        <v>0</v>
+      </c>
+      <c r="O38" s="16">
+        <v>0</v>
+      </c>
+      <c r="P38" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="16">
+        <v>0</v>
+      </c>
+      <c r="R38" s="16">
+        <v>0</v>
+      </c>
+      <c r="S38" s="16">
+        <v>0</v>
+      </c>
+      <c r="T38" s="16">
+        <v>0</v>
+      </c>
+      <c r="U38" s="16">
+        <v>0</v>
+      </c>
+      <c r="V38" s="16">
+        <v>0</v>
+      </c>
+      <c r="W38" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" ht="48.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B39" s="34" t="s">
+        <v>124</v>
+      </c>
+      <c r="C39" s="34" t="s">
+        <v>125</v>
+      </c>
+      <c r="D39" s="49">
+        <v>46250</v>
+      </c>
+      <c r="E39" s="13">
+        <v>46251</v>
+      </c>
+      <c r="F39" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G39" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="H39" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I39" s="15">
+        <v>5</v>
+      </c>
+      <c r="J39" s="15">
+        <v>1</v>
+      </c>
+      <c r="K39" s="15">
+        <v>1</v>
+      </c>
+      <c r="L39" s="15">
+        <v>1</v>
+      </c>
+      <c r="M39" s="16">
+        <v>1</v>
+      </c>
+      <c r="N39" s="16">
+        <v>1</v>
+      </c>
+      <c r="O39" s="16">
+        <v>0</v>
+      </c>
+      <c r="P39" s="16">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="16">
+        <v>0</v>
+      </c>
+      <c r="R39" s="16">
+        <v>0</v>
+      </c>
+      <c r="S39" s="16">
+        <v>0</v>
+      </c>
+      <c r="T39" s="16">
+        <v>0</v>
+      </c>
+      <c r="U39" s="16">
+        <v>0</v>
+      </c>
+      <c r="V39" s="16">
+        <v>0</v>
+      </c>
+      <c r="W39" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="32" t="s">
+        <v>126</v>
+      </c>
+      <c r="B40" s="34" t="s">
+        <v>127</v>
+      </c>
+      <c r="C40" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="D40" s="49">
+        <v>46249</v>
+      </c>
+      <c r="E40" s="13">
+        <v>46251</v>
+      </c>
+      <c r="F40" s="44" t="s">
+        <v>28</v>
+      </c>
+      <c r="G40" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="H40" s="44" t="s">
+        <v>30</v>
+      </c>
+      <c r="I40" s="15">
+        <v>8</v>
+      </c>
+      <c r="J40" s="15">
+        <v>1</v>
+      </c>
+      <c r="K40" s="15">
+        <v>1</v>
+      </c>
+      <c r="L40" s="15">
+        <v>1</v>
+      </c>
+      <c r="M40" s="16">
+        <v>1</v>
+      </c>
+      <c r="N40" s="16">
+        <v>1</v>
+      </c>
+      <c r="O40" s="16">
+        <v>1</v>
+      </c>
+      <c r="P40" s="16">
+        <v>1</v>
+      </c>
+      <c r="Q40" s="16">
+        <v>1</v>
+      </c>
+      <c r="R40" s="16">
+        <v>0</v>
+      </c>
+      <c r="S40" s="16">
+        <v>0</v>
+      </c>
+      <c r="T40" s="16">
+        <v>0</v>
+      </c>
+      <c r="U40" s="16">
+        <v>0</v>
+      </c>
+      <c r="V40" s="16">
+        <v>0</v>
+      </c>
+      <c r="W40" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:23" ht="17.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="49" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="50" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="51" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3972,13 +5376,14 @@
     <row r="106" ht="22.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection password="E403" sheet="1" objects="1" scenarios="1" formatCells="0" formatRows="0" insertRows="0" deleteRows="0"/>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A18:W18"/>
+    <mergeCell ref="A27:W27"/>
     <mergeCell ref="A4:W4"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="A11:W11"/>
+    <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="E2:E3"/>
@@ -4015,26 +5420,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="46" customWidth="1"/>
-    <col min="4" max="4" width="56.88671875" customWidth="1"/>
+    <col min="3" max="3" width="72.77734375" customWidth="1"/>
+    <col min="4" max="4" width="80.33203125" customWidth="1"/>
     <col min="5" max="5" width="33.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>123</v>
+        <v>169</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>124</v>
+        <v>170</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>125</v>
+        <v>171</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>126</v>
+        <v>172</v>
       </c>
       <c r="E1" s="8"/>
       <c r="F1" s="8"/>
@@ -4042,156 +5447,254 @@
     </row>
     <row r="2" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>127</v>
+        <v>173</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>128</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>130</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>131</v>
+        <v>177</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>132</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="B5" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>133</v>
+        <v>179</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>134</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>136</v>
+        <v>182</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>137</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>138</v>
+        <v>184</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>139</v>
+        <v>185</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>140</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>141</v>
+        <v>187</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>142</v>
+        <v>188</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>143</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>144</v>
+        <v>190</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>145</v>
+        <v>191</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>146</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>147</v>
+        <v>193</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>148</v>
+        <v>194</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>149</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>150</v>
+        <v>196</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>151</v>
+        <v>197</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>152</v>
+        <v>198</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>155</v>
+        <v>201</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -4203,47 +5706,47 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.88671875" style="1" customWidth="1"/>
     <col min="2" max="4" width="12.33203125" style="3" customWidth="1"/>
     <col min="5" max="5" width="20.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="53.33203125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="27.33203125" style="4" customWidth="1"/>
-    <col min="8" max="8" width="38.77734375" style="1" customWidth="1"/>
-    <col min="9" max="9" width="42.33203125" style="1" customWidth="1"/>
-    <col min="10" max="18" width="9.109375" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="9.109375" style="1"/>
+    <col min="6" max="6" width="64" style="3" customWidth="1"/>
+    <col min="7" max="7" width="40.77734375" style="4" customWidth="1"/>
+    <col min="8" max="8" width="59" style="1" customWidth="1"/>
+    <col min="9" max="9" width="76.5546875" style="1" customWidth="1"/>
+    <col min="10" max="20" width="9.109375" style="1" customWidth="1"/>
+    <col min="21" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="2" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>156</v>
+        <v>216</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>157</v>
+        <v>217</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>158</v>
+        <v>218</v>
       </c>
       <c r="D1" s="20" t="s">
-        <v>159</v>
+        <v>219</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="F1" s="20" t="s">
-        <v>161</v>
+        <v>221</v>
       </c>
       <c r="G1" s="20" t="s">
-        <v>162</v>
+        <v>222</v>
       </c>
       <c r="H1" s="20" t="s">
-        <v>163</v>
+        <v>223</v>
       </c>
       <c r="I1" s="20" t="s">
-        <v>164</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -4251,7 +5754,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C2" s="30">
         <v>46204</v>
@@ -4259,20 +5762,20 @@
       <c r="D2" s="30">
         <v>46216</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="53" t="s">
         <v>28</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>165</v>
+        <v>225</v>
       </c>
       <c r="G2" s="55" t="s">
-        <v>166</v>
+        <v>226</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>167</v>
+        <v>227</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>168</v>
+        <v>228</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -4280,7 +5783,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="C3" s="30">
         <v>46204</v>
@@ -4292,16 +5795,16 @@
         <v>28</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>169</v>
+        <v>229</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>171</v>
+        <v>231</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>172</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -4309,7 +5812,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C4" s="30">
         <v>46217</v>
@@ -4321,16 +5824,16 @@
         <v>28</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>173</v>
+        <v>233</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>174</v>
+        <v>234</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>175</v>
+        <v>235</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>176</v>
+        <v>236</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -4338,7 +5841,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C5" s="30">
         <v>46217</v>
@@ -4350,16 +5853,16 @@
         <v>28</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>177</v>
+        <v>237</v>
       </c>
       <c r="G5" s="55" t="s">
-        <v>178</v>
+        <v>238</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>179</v>
+        <v>239</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>180</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -4367,7 +5870,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C6" s="30">
         <v>46217</v>
@@ -4379,16 +5882,16 @@
         <v>28</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>181</v>
+        <v>241</v>
       </c>
       <c r="G6" s="55" t="s">
-        <v>182</v>
+        <v>242</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>183</v>
+        <v>243</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>184</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -4396,7 +5899,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C7" s="30">
         <v>46217</v>
@@ -4408,16 +5911,16 @@
         <v>28</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>185</v>
+        <v>245</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>186</v>
+        <v>246</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>187</v>
+        <v>247</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>188</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -4425,7 +5928,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>109</v>
+        <v>145</v>
       </c>
       <c r="C8" s="30">
         <v>46217</v>
@@ -4437,16 +5940,16 @@
         <v>28</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>189</v>
+        <v>249</v>
       </c>
       <c r="G8" s="55" t="s">
-        <v>190</v>
+        <v>250</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>191</v>
+        <v>251</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>192</v>
+        <v>252</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -4454,7 +5957,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C9" s="30">
         <v>46231</v>
@@ -4466,16 +5969,16 @@
         <v>28</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>193</v>
+        <v>253</v>
       </c>
       <c r="G9" s="55" t="s">
-        <v>194</v>
+        <v>254</v>
       </c>
       <c r="H9" s="53" t="s">
-        <v>195</v>
+        <v>255</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>196</v>
+        <v>256</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -4483,7 +5986,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C10" s="30">
         <v>46236</v>
@@ -4495,16 +5998,16 @@
         <v>28</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>197</v>
+        <v>257</v>
       </c>
       <c r="G10" s="55" t="s">
-        <v>198</v>
+        <v>258</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>199</v>
+        <v>259</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>200</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
@@ -4512,7 +6015,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>116</v>
+        <v>152</v>
       </c>
       <c r="C11" s="30">
         <v>46207</v>
@@ -4524,16 +6027,103 @@
         <v>28</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>201</v>
+        <v>261</v>
       </c>
       <c r="G11" s="55" t="s">
-        <v>202</v>
+        <v>262</v>
       </c>
       <c r="H11" s="53" t="s">
-        <v>203</v>
+        <v>263</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>204</v>
+        <v>264</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>12</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C12" s="30">
+        <v>46240</v>
+      </c>
+      <c r="D12" s="30">
+        <v>46244</v>
+      </c>
+      <c r="E12" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="G12" s="55" t="s">
+        <v>266</v>
+      </c>
+      <c r="H12" s="53" t="s">
+        <v>267</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>13</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" s="30">
+        <v>46244</v>
+      </c>
+      <c r="D13" s="30">
+        <v>46247</v>
+      </c>
+      <c r="E13" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="G13" s="55" t="s">
+        <v>270</v>
+      </c>
+      <c r="H13" s="53" t="s">
+        <v>271</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="26.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>14</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C14" s="30">
+        <v>46248</v>
+      </c>
+      <c r="D14" s="30">
+        <v>46250</v>
+      </c>
+      <c r="E14" s="53" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="G14" s="55" t="s">
+        <v>274</v>
+      </c>
+      <c r="H14" s="53" t="s">
+        <v>275</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>276</v>
       </c>
     </row>
   </sheetData>

</xml_diff>